<commit_message>
Mudança no dicionário de dados: mudança de mySQL para SQL por questões de organização, correção com o role sendo separado ('cliente', 'admin').
</commit_message>
<xml_diff>
--- a/docs/Dicionario_Dados_ClubePlanner.xlsx
+++ b/docs/Dicionario_Dados_ClubePlanner.xlsx
@@ -989,8 +989,10 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t>Tipo (SQLite)</t>
+        </is>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -1025,8 +1027,10 @@
       <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>10</v>
+      <c r="C3" t="inlineStr" s="3">
+        <is>
+          <t>INTEGER PRIMARY KEY AUTOINCREMENT</t>
+        </is>
       </c>
       <c r="D3" s="3" t="s">
         <v>11</v>
@@ -1047,8 +1051,10 @@
       <c r="B4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>16</v>
+      <c r="C4" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="5" t="s">
@@ -1067,8 +1073,10 @@
       <c r="B5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>19</v>
+      <c r="C5" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D5" s="5" t="s">
         <v>20</v>
@@ -1089,8 +1097,10 @@
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>23</v>
+      <c r="C6" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
@@ -1109,8 +1119,10 @@
       <c r="B7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>26</v>
+      <c r="C7" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D7" s="5" t="s">
         <v>20</v>
@@ -1131,8 +1143,10 @@
       <c r="B8" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>29</v>
+      <c r="C8" t="inlineStr" s="5">
+        <is>
+          <t>TEXT CHECK (role IN ('client','admin'))</t>
+        </is>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5" t="s">
@@ -1151,15 +1165,19 @@
       <c r="B9" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>33</v>
+      <c r="C9" t="inlineStr" s="5">
+        <is>
+          <t>TEXT (ISO8601, default datetime('now'))</t>
+        </is>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>34</v>
+      <c r="F9" t="inlineStr" s="5">
+        <is>
+          <t>datetime('now')</t>
+        </is>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="6" t="s">
@@ -1183,8 +1201,10 @@
       <c r="B11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>10</v>
+      <c r="C11" t="inlineStr" s="3">
+        <is>
+          <t>INTEGER PRIMARY KEY AUTOINCREMENT</t>
+        </is>
       </c>
       <c r="D11" s="3" t="s">
         <v>11</v>
@@ -1205,8 +1225,10 @@
       <c r="B12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>39</v>
+      <c r="C12" t="inlineStr" s="7">
+        <is>
+          <t>INTEGER</t>
+        </is>
       </c>
       <c r="D12" s="7" t="s">
         <v>40</v>
@@ -1229,8 +1251,10 @@
       <c r="B13" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>44</v>
+      <c r="C13" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5" t="s">
@@ -1249,8 +1273,10 @@
       <c r="B14" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>47</v>
+      <c r="C14" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5" t="s">
@@ -1269,8 +1295,10 @@
       <c r="B15" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>50</v>
+      <c r="C15" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5" t="s">
@@ -1289,8 +1317,10 @@
       <c r="B16" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>53</v>
+      <c r="C16" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5" t="s">
@@ -1309,8 +1339,10 @@
       <c r="B17" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="5" t="s">
-        <v>53</v>
+      <c r="C17" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="5" t="s">
@@ -1349,8 +1381,10 @@
       <c r="B19" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>63</v>
+      <c r="C19" t="inlineStr" s="5">
+        <is>
+          <t>INTEGER (0/1)</t>
+        </is>
       </c>
       <c r="D19" s="5"/>
       <c r="E19" s="5" t="s">
@@ -1381,8 +1415,10 @@
       <c r="B21" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>10</v>
+      <c r="C21" t="inlineStr" s="3">
+        <is>
+          <t>INTEGER PRIMARY KEY AUTOINCREMENT</t>
+        </is>
       </c>
       <c r="D21" s="3" t="s">
         <v>11</v>
@@ -1403,8 +1439,10 @@
       <c r="B22" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C22" s="5" t="s">
-        <v>53</v>
+      <c r="C22" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D22" s="5"/>
       <c r="E22" s="5" t="s">
@@ -1423,8 +1461,10 @@
       <c r="B23" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>70</v>
+      <c r="C23" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D23" s="5" t="s">
         <v>20</v>
@@ -1457,8 +1497,10 @@
       <c r="B25" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>10</v>
+      <c r="C25" t="inlineStr" s="3">
+        <is>
+          <t>INTEGER PRIMARY KEY AUTOINCREMENT</t>
+        </is>
       </c>
       <c r="D25" s="3" t="s">
         <v>11</v>
@@ -1479,8 +1521,10 @@
       <c r="B26" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="C26" s="7" t="s">
-        <v>39</v>
+      <c r="C26" t="inlineStr" s="7">
+        <is>
+          <t>INTEGER</t>
+        </is>
       </c>
       <c r="D26" s="7" t="s">
         <v>40</v>
@@ -1503,8 +1547,10 @@
       <c r="B27" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C27" s="5" t="s">
-        <v>19</v>
+      <c r="C27" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D27" s="5"/>
       <c r="E27" s="5" t="s">
@@ -1543,8 +1589,10 @@
       <c r="B29" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C29" s="5" t="s">
-        <v>82</v>
+      <c r="C29" t="inlineStr" s="5">
+        <is>
+          <t>REAL</t>
+        </is>
       </c>
       <c r="D29" s="5"/>
       <c r="E29" s="5" t="s">
@@ -1563,8 +1611,10 @@
       <c r="B30" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>39</v>
+      <c r="C30" t="inlineStr" s="5">
+        <is>
+          <t>INTEGER</t>
+        </is>
       </c>
       <c r="D30" s="5"/>
       <c r="E30" s="5" t="s">
@@ -1583,8 +1633,10 @@
       <c r="B31" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C31" s="5" t="s">
-        <v>63</v>
+      <c r="C31" t="inlineStr" s="5">
+        <is>
+          <t>INTEGER (0/1)</t>
+        </is>
       </c>
       <c r="D31" s="5"/>
       <c r="E31" s="5" t="s">
@@ -1615,8 +1667,10 @@
       <c r="B33" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C33" s="3" t="s">
-        <v>10</v>
+      <c r="C33" t="inlineStr" s="3">
+        <is>
+          <t>INTEGER PRIMARY KEY AUTOINCREMENT</t>
+        </is>
       </c>
       <c r="D33" s="3" t="s">
         <v>11</v>
@@ -1637,8 +1691,10 @@
       <c r="B34" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C34" s="7" t="s">
-        <v>39</v>
+      <c r="C34" t="inlineStr" s="7">
+        <is>
+          <t>INTEGER</t>
+        </is>
       </c>
       <c r="D34" s="7" t="s">
         <v>40</v>
@@ -1661,8 +1717,10 @@
       <c r="B35" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="C35" s="7" t="s">
-        <v>39</v>
+      <c r="C35" t="inlineStr" s="7">
+        <is>
+          <t>INTEGER</t>
+        </is>
       </c>
       <c r="D35" s="7" t="s">
         <v>40</v>
@@ -1685,8 +1743,10 @@
       <c r="B36" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="C36" s="5" t="s">
-        <v>96</v>
+      <c r="C36" t="inlineStr" s="5">
+        <is>
+          <t>TEXT CHECK (status IN ('pending','paid','shipped','delivered','canceled'))</t>
+        </is>
       </c>
       <c r="D36" s="5"/>
       <c r="E36" s="5" t="s">
@@ -1705,8 +1765,10 @@
       <c r="B37" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="C37" s="5" t="s">
-        <v>82</v>
+      <c r="C37" t="inlineStr" s="5">
+        <is>
+          <t>REAL</t>
+        </is>
       </c>
       <c r="D37" s="5"/>
       <c r="E37" s="5" t="s">
@@ -1725,8 +1787,10 @@
       <c r="B38" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="C38" s="5" t="s">
-        <v>82</v>
+      <c r="C38" t="inlineStr" s="5">
+        <is>
+          <t>REAL</t>
+        </is>
       </c>
       <c r="D38" s="5"/>
       <c r="E38" s="5" t="s">
@@ -1745,15 +1809,19 @@
       <c r="B39" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C39" s="5" t="s">
-        <v>33</v>
+      <c r="C39" t="inlineStr" s="5">
+        <is>
+          <t>TEXT (ISO8601, default datetime('now'))</t>
+        </is>
       </c>
       <c r="D39" s="5"/>
       <c r="E39" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F39" s="5" t="s">
-        <v>34</v>
+      <c r="F39" t="inlineStr" s="5">
+        <is>
+          <t>datetime('now')</t>
+        </is>
       </c>
       <c r="G39" s="5"/>
       <c r="H39" s="6" t="s">
@@ -1777,8 +1845,10 @@
       <c r="B41" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C41" s="3" t="s">
-        <v>10</v>
+      <c r="C41" t="inlineStr" s="3">
+        <is>
+          <t>INTEGER PRIMARY KEY AUTOINCREMENT</t>
+        </is>
       </c>
       <c r="D41" s="3" t="s">
         <v>11</v>
@@ -1799,8 +1869,10 @@
       <c r="B42" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C42" s="7" t="s">
-        <v>39</v>
+      <c r="C42" t="inlineStr" s="7">
+        <is>
+          <t>INTEGER</t>
+        </is>
       </c>
       <c r="D42" s="7" t="s">
         <v>40</v>
@@ -1823,8 +1895,10 @@
       <c r="B43" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="C43" s="7" t="s">
-        <v>39</v>
+      <c r="C43" t="inlineStr" s="7">
+        <is>
+          <t>INTEGER</t>
+        </is>
       </c>
       <c r="D43" s="7" t="s">
         <v>40</v>
@@ -1847,8 +1921,10 @@
       <c r="B44" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C44" s="5" t="s">
-        <v>39</v>
+      <c r="C44" t="inlineStr" s="5">
+        <is>
+          <t>INTEGER</t>
+        </is>
       </c>
       <c r="D44" s="5"/>
       <c r="E44" s="5" t="s">
@@ -1867,8 +1943,10 @@
       <c r="B45" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="C45" s="5" t="s">
-        <v>82</v>
+      <c r="C45" t="inlineStr" s="5">
+        <is>
+          <t>REAL</t>
+        </is>
       </c>
       <c r="D45" s="5"/>
       <c r="E45" s="5" t="s">
@@ -1899,8 +1977,10 @@
       <c r="B47" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C47" s="3" t="s">
-        <v>10</v>
+      <c r="C47" t="inlineStr" s="3">
+        <is>
+          <t>INTEGER PRIMARY KEY AUTOINCREMENT</t>
+        </is>
       </c>
       <c r="D47" s="3" t="s">
         <v>11</v>
@@ -1921,8 +2001,10 @@
       <c r="B48" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C48" s="7" t="s">
-        <v>39</v>
+      <c r="C48" t="inlineStr" s="7">
+        <is>
+          <t>INTEGER</t>
+        </is>
       </c>
       <c r="D48" s="7" t="s">
         <v>40</v>
@@ -1945,8 +2027,10 @@
       <c r="B49" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="C49" s="5" t="s">
-        <v>121</v>
+      <c r="C49" t="inlineStr" s="5">
+        <is>
+          <t>TEXT CHECK (metodo IN ('pix','cartao','boleto'))</t>
+        </is>
       </c>
       <c r="D49" s="5"/>
       <c r="E49" s="5" t="s">
@@ -1965,8 +2049,10 @@
       <c r="B50" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="C50" s="5" t="s">
-        <v>124</v>
+      <c r="C50" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D50" s="5"/>
       <c r="E50" s="5" t="s">
@@ -1985,8 +2071,10 @@
       <c r="B51" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="C51" s="5" t="s">
-        <v>53</v>
+      <c r="C51" t="inlineStr" s="5">
+        <is>
+          <t>TEXT</t>
+        </is>
       </c>
       <c r="D51" s="5"/>
       <c r="E51" s="5" t="s">
@@ -2005,15 +2093,19 @@
       <c r="B52" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="C52" s="5" t="s">
-        <v>33</v>
+      <c r="C52" t="inlineStr" s="5">
+        <is>
+          <t>TEXT (ISO8601, default datetime('now'))</t>
+        </is>
       </c>
       <c r="D52" s="5"/>
       <c r="E52" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F52" s="5" t="s">
-        <v>34</v>
+      <c r="F52" t="inlineStr" s="5">
+        <is>
+          <t>datetime('now')</t>
+        </is>
       </c>
       <c r="G52" s="5"/>
       <c r="H52" s="6" t="s">

</xml_diff>